<commit_message>
Refresh the 13 Sep Google News screen and compare it with August snapshots.
Fall back to News RSS when the HTML SERP is rate-limited, match cards by article id/title, and publish an Excel workbook with analytics and three-run position trends.

Co-authored-by: Ilya Rost <jaguarcatcat@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/aktualnaya_vydacha.xlsx
+++ b/output/aktualnaya_vydacha.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Выдача" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Выдача'!$A$1:$J$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Выдача'!$A$1:$J$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,14 +446,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
@@ -531,12 +531,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Sostav.ru</t>
+          <t>sostav.ru</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13 00:04 MSK</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -578,17 +578,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-20 11:00 MSK</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -598,12 +598,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия, университет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -630,17 +630,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>zarya-egorlik.ru</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2025-11-01 10:00 MSK</t>
+          <t>Tue, 20 Jan 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>zarya-egorlik.ru</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия, университет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00 MSK</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -734,17 +734,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2024-07-12 15:04 MSK</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -754,22 +754,22 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -786,17 +786,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: предприниматель и создатель «Синергии»</t>
+          <t>Вадим Лобов — обо мне</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Вести Подмосковья</t>
+          <t>Сноб</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2024-05-28 10:00 MSK</t>
+          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -806,12 +806,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://vmo24.ru/news/vadim_lobov_predprinimatel_i_sozdatel_sinergii</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>vmo24.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
         </is>
       </c>
     </row>
@@ -838,17 +838,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Проект медиа</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2018-10-22 10:00 MSK</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -858,22 +858,22 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>proekt.media</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>расследование</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -890,17 +890,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Проект медиа</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2024-02-03 11:00 MSK</t>
+          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -910,22 +910,22 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>proekt.media</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>расследование</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
         </is>
       </c>
     </row>
@@ -942,17 +942,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>Интервью с президентом «Синергии»: «Будем привлекать молодежь к правовому просвещению школьников» - новости Право.ру</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>SakhaDay</t>
+          <t>ПРАВО.Ru</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2024-08-12 10:00 MSK</t>
+          <t>Fri, 05 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -962,22 +962,22 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://pravo.ru/story/253963/</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>pravo.ru</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>интервью</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
         </is>
       </c>
     </row>
@@ -994,17 +994,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>С Днём рождения, Вадим Лобов!</t>
+          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Союз ММА России</t>
+          <t>Парламент.UA</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2021-08-02 10:00 MSK</t>
+          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://mmaunion.ru/news/s-dnyom-rozhdeniya-vadim-lobov/</t>
+          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>mmaunion.ru</t>
+          <t>parlament.ua</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>досье / биография</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1046,17 +1046,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Глава «Синергии» Вадим Лобов объявил о запуске программ двойного диплома с вузами Сербии</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2022-08-31 10:00 MSK</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2022/08/31/universitet-sinergiya-serbua/</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
         </is>
       </c>
     </row>
@@ -1098,17 +1098,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
+          <t>Вадим Георгиевич Лобов: Наши студенты смогут получить два диплома — «Синергии» и ведущего университета страны БРИКС | Россия-Онлайн- новости России</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Парламент.UA</t>
+          <t>russia-on.ru</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2024-07-18 10:00 MSK</t>
+          <t>Mon, 12 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1118,22 +1118,22 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
+          <t>https://news.google.com/rss/articles/CBMiRkFVX3lxTE5rTkNqaHYwV0NDQjUtQVRrazJ4SFV0OXM5dmYzVTctWUxPdzRCc284YVFsM0o4YjBkOFJKY090c3pVbDF3NHc?oc=5</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>parlament.ua</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>досье / биография</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1150,17 +1150,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов: Наши студенты смогут получить два диплома — «Синергии» и ведущего университета страны БРИКС | Россия-Онлайн</t>
+          <t>Глава «Синергии» Вадим Лобов анонсировал запуск Центра трансфера технологий для превращения инноваций в бизнес-продукты — Осетия ТВ</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>russia-on.ru</t>
+          <t>Осетия ТВ</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2024-02-12 11:00 MSK</t>
+          <t>Tue, 07 Mar 2023 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1170,22 +1170,22 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>http://www.russia-on.ru/184386</t>
+          <t>https://www.ossetia.tv/2023/03/07/lobov-vadim-georgievich-universiteta-sinergiya/</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>russia-on.ru</t>
+          <t>ossetia.tv</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -1202,17 +1202,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Друзья Шварценеггера: Как владельцы университета "Синергия" зарабатывают миллиарды</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2022-10-24 10:00 MSK</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1222,12 +1222,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>https://m.repost.news/news/9867-druzjja_shvartseneggera_kak_vladeljtsy_universiteta_sinergija_zarabatyvajut_milliardy/print</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>m.repost.news</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия, университет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -1254,17 +1254,17 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Глава «Синергии» Вадим Лобов пригласил участников ВФМ-2024 стать амбассадорами российского образования за рубежом — Осетия ТВ</t>
+          <t>Мошенничество под прикрытием ВУЗа: как разводят на деньги студентов «Синергии»</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2024-03-09 11:00 MSK</t>
+          <t>Tue, 15 Nov 2022 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2024/03/09/glava-sinergii-vadim-lobov-priglasil-uchastnikov-vfm-2024-stat-ambassadorami-rossijskogo-obrazovaniya-za-rubezhom/</t>
+          <t>https://repost.news/news/11272-moshennichestvo_pod_prikrytiem_vuza_kak_razvodjat_na_denjgi_studentov_sinergii</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1289,34 +1289,34 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим университет синергия</t>
+          <t>лобов вадим синергия</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Глава «Синергии» Вадим Лобов анонсировал запуск Центра трансфера технологий для превращения инноваций в бизнес-продукты — Осетия ТВ</t>
+          <t>Вадим Георгиевич Лобов и корпорация "Синергия" в фокусе внимания моего очередного подкаста ЖЗЛ Ростокин. Digital</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>sostav.ru</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2023-03-07 11:00 MSK</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1326,49 +1326,49 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2023/03/07/lobov-vadim-georgievich-universiteta-sinergiya/</t>
+          <t>https://www.sostav.ru/blogs/289047/94470</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>sostav.ru</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>блог / колонка / подкаст</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим университет синергия</t>
+          <t>лобов вадим синергия</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Мошенничество под прикрытием ВУЗа: как разводят на деньги студентов «Синергии»</t>
+          <t>Президент «Синергии» Лобов: «Грамотная миграционная политика—решение проблемы кадров»</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2022-11-15 11:00 MSK</t>
+          <t>Mon, 29 Dec 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1378,12 +1378,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/11272-moshennichestvo_pod_prikrytiem_vuza_kak_razvodjat_na_denjgi_studentov_sinergii</t>
+          <t>https://www.forbes.ru/club/552791-prezident-sinergii-lobov-gramotnaa-migracionnaa-politika-resenie-problemy-kadrov</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
+          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
         </is>
       </c>
     </row>
@@ -1405,22 +1405,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов и корпорация "Синергия" в фокусе внимания моего очередного подкаста ЖЗЛ Ростокин. Digital</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Sostav.ru</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13 00:04 MSK</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1430,17 +1430,17 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>https://www.sostav.ru/blogs/289047/94470</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>блог / колонка / подкаст</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1457,22 +1457,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Президент «Синергии» Лобов: «Грамотная миграционная политика—решение проблемы кадров»</t>
+          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Forbes.ru</t>
+          <t>Журнал ФОМА</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2025-12-29 11:00 MSK</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1482,12 +1482,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>https://www.forbes.ru/club/552791-prezident-sinergii-lobov-gramotnaa-migracionnaa-politika-resenie-problemy-kadrov</t>
+          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>forbes.ru</t>
+          <t>foma.ru</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
         </is>
       </c>
     </row>
@@ -1509,22 +1509,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
+          <t>Президент «Синергии» Лобов представил патриарху Кириллу проект экотроп на Валааме</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Журнал ФОМА</t>
+          <t>Общественная служба новостей</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15 10:00 MSK</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPS3ZGa1N3RGN2aU9yRkxpT3NKb2Z3RFJ4b3VjbWl6S3V2QmxDU2FSbng3eUdoWm1kQk9OMnNmbU9JeTcxX3VtNC1OSExJTGQ3UllKYkZRZnYtM2kxVV9NOUZ1TFZRNnNmNVdtc3Vnd2k1bzVSeTRxWmFJVGhLY0dpUWhxaVN3cG1nb0Q0b3hDOUhlUmV6RVgxRTlBRmQ2aDd3N21USGJ3X280dXdqRlNoeHFKdzgtZw?oc=5</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>foma.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
+          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
         </is>
       </c>
     </row>
@@ -1561,22 +1561,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>SMINEWS</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2025-11-01 10:00 MSK</t>
+          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1586,12 +1586,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://sminews.ru/2891</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>sminews.ru</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1613,22 +1613,22 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
+          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>SMINEWS</t>
+          <t>zarya-egorlik.ru</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2025-11-03 11:00 MSK</t>
+          <t>Tue, 20 Jan 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1638,22 +1638,22 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>https://sminews.ru/2891</t>
+          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>sminews.ru</t>
+          <t>zarya-egorlik.ru</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1665,22 +1665,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
+          <t>Вадим Лобов — обо мне</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>Сноб</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-01-20 11:00 MSK</t>
+          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00 MSK</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1769,22 +1769,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2024-07-12 15:04 MSK</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -1821,22 +1821,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: предприниматель и создатель «Синергии»</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Вести Подмосковья</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2024-05-28 10:00 MSK</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1846,12 +1846,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>https://vmo24.ru/news/vadim_lobov_predprinimatel_i_sozdatel_sinergii</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>vmo24.ru</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1873,22 +1873,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Интервью с президентом «Синергии»: «Будем привлекать молодежь к правовому просвещению школьников» - новости Право.ру</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>ПРАВО.Ru</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2024-02-03 11:00 MSK</t>
+          <t>Fri, 05 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1898,22 +1898,22 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://pravo.ru/story/253963/</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>pravo.ru</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>интервью</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1925,22 +1925,22 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>С Днём рождения, Вадим Лобов!</t>
+          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Союз ММА России</t>
+          <t>Проект медиа</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2021-08-02 10:00 MSK</t>
+          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1950,22 +1950,22 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://mmaunion.ru/news/s-dnyom-rozhdeniya-vadim-lobov/</t>
+          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>mmaunion.ru</t>
+          <t>proekt.media</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>расследование</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1987,12 +1987,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>SakhaDay</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2024-08-12 10:00 MSK</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2029,22 +2029,22 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
+          <t>Рост EdTech-выручки «Синергии» трехкратно превысил средний показатель рынка</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>TAdviser</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2025-09-10 10:00 MSK</t>
+          <t>Fri, 26 Apr 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2054,12 +2054,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
+          <t>https://www.tadviser.ru/index.php/%D0%9A%D0%BE%D0%BC%D0%BF%D0%B0%D0%BD%D0%B8%D1%8F:%D0%A1%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F_%D0%9A%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>tadviser.ru</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2081,22 +2081,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
+          <t>Предновогодний гала-вечер «Хрустальная симфония» Корпорации «Синергия» и Posta-Magazine</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Проект медиа</t>
+          <t>Posta-Magazine</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2018-10-22 10:00 MSK</t>
+          <t>Mon, 16 Dec 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2106,17 +2106,17 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
+          <t>https://posta-magazine.ru/article/khrustalnaya-simfonia-2024/</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>proekt.media</t>
+          <t>posta-magazine.ru</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>расследование</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2133,22 +2133,22 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>«Синергия» и Право.ru договорились развивать правовую культуру РФ - новости Право.ру</t>
+          <t>Елизавета Фролова: «Я вижу тренд на возвращение академического искусства»</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>ПРАВО.Ru</t>
+          <t>The Art Newspaper Russia</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2023-05-11 10:00 MSK</t>
+          <t>Thu, 18 Sep 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>https://pravo.ru/lf/news/246443/</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9SX0U3RnB1SmQteFRTNVZJdkRUNmZWWkZlVTdiYUYyUVNMcFdhSFVab1dGa1gzNllPUXdEczRMMnhEeFVGM3I4TkU3Mk05bDk2RU94T21vX2dOU2huVWwxZQ?oc=5</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>pravo.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов: Наши студенты смогут получить два диплома — «Синергии» и ведущего университета страны БРИКС | Россия-Онлайн</t>
+          <t>Корпорация «Синергия» приобрела часть российского бизнеса международной группы Hays</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>russia-on.ru</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2024-02-12 11:00 MSK</t>
+          <t>Wed, 27 Jul 2022 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2210,12 +2210,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>http://www.russia-on.ru/184386</t>
+          <t>https://www.forbes.ru/svoi-biznes/472819-korporacia-sinergia-priobrela-cast-rossijskogo-biznesa-mezdunarodnoj-gruppy-hays</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>russia-on.ru</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2237,22 +2237,22 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Рост EdTech-выручки «Синергии» трехкратно превысил средний показатель рынка</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>TAdviser</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2024-04-26 10:00 MSK</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2262,12 +2262,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>https://www.tadviser.ru/index.php/%D0%9A%D0%BE%D0%BC%D0%BF%D0%B0%D0%BD%D0%B8%D1%8F:%D0%A1%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F_%D0%9A%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>tadviser.ru</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Друзья Шварценеггера: Как владельцы университета "Синергия" зарабатывают миллиарды</t>
+          <t>Вадим Георгиевич Лобов: Наши студенты смогут получить два диплома — «Синергии» и ведущего университета страны БРИКС | Россия-Онлайн- новости России</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>russia-on.ru</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2022-10-24 10:00 MSK</t>
+          <t>Mon, 12 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2314,12 +2314,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>https://m.repost.news/news/9867-druzjja_shvartseneggera_kak_vladeljtsy_universiteta_sinergija_zarabatyvajut_milliardy/print</t>
+          <t>https://news.google.com/rss/articles/CBMiRkFVX3lxTE5rTkNqaHYwV0NDQjUtQVRrazJ4SFV0OXM5dmYzVTctWUxPdzRCc284YVFsM0o4YjBkOFJKY090c3pVbDF3NHc?oc=5</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>m.repost.news</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2329,34 +2329,34 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим синергия</t>
+          <t>лобов вадим</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Глава «Синергии» Вадим Лобов пригласил участников ВФМ-2024 стать амбассадорами российского образования за рубежом — Осетия ТВ</t>
+          <t>Вадим Георгиевич Лобов и корпорация "Синергия" в фокусе внимания моего очередного подкаста ЖЗЛ Ростокин. Digital</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>sostav.ru</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2024-03-09 11:00 MSK</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2366,49 +2366,49 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2024/03/09/glava-sinergii-vadim-lobov-priglasil-uchastnikov-vfm-2024-stat-ambassadorami-rossijskogo-obrazovaniya-za-rubezhom/</t>
+          <t>https://www.sostav.ru/blogs/289047/94470</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>sostav.ru</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>блог / колонка / подкаст</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим синергия</t>
+          <t>лобов вадим</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Глава «Синергии» Вадим Лобов объявил о запуске программ двойного диплома с вузами Сербии</t>
+          <t>Основатели «Арт России» Вадим Лобов и Елизавета Фролова — о коллекционировании без посредников</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>buro247.ru</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2022-08-31 10:00 MSK</t>
+          <t>Fri, 27 Mar 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2022/08/31/universitet-sinergiya-serbua/</t>
+          <t>https://www.buro247.ru/culture/arts/23-mar-2026-art-russia-interview.html</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>buro247.ru</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов и корпорация "Синергия" в фокусе внимания моего очередного подкаста ЖЗЛ Ростокин. Digital</t>
+          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Sostav.ru</t>
+          <t>Журнал ФОМА</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13 00:04 MSK</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2470,22 +2470,22 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>https://www.sostav.ru/blogs/289047/94470</t>
+          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>foma.ru</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>блог / колонка / подкаст</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2497,22 +2497,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Основатели «Арт России» Вадим Лобов и Елизавета Фролова — о коллекционировании без посредников</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>buro247.ru</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-03-27 10:00 MSK</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2522,12 +2522,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>https://www.buro247.ru/culture/arts/23-mar-2026-art-russia-interview.html</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>buro247.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2549,22 +2549,22 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
+          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Журнал ФОМА</t>
+          <t>SMINEWS</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15 10:00 MSK</t>
+          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2574,22 +2574,22 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
+          <t>https://sminews.ru/2891</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>foma.ru</t>
+          <t>sminews.ru</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2601,22 +2601,22 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Вадим Лобов — обо мне</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>Сноб</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2025-11-01 10:00 MSK</t>
+          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2626,17 +2626,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -2653,22 +2653,22 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
+          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>SMINEWS</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2025-11-03 11:00 MSK</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2678,17 +2678,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>https://sminews.ru/2891</t>
+          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>sminews.ru</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -2705,22 +2705,22 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00 MSK</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2730,17 +2730,17 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03 10:00 MSK</t>
+          <t>Fri, 03 Apr 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2024-07-12 15:04 MSK</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2861,22 +2861,22 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: предприниматель и создатель «Синергии»</t>
+          <t>Корпорация «Синергия» приобрела часть российского бизнеса международной группы Hays</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Вести Подмосковья</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2024-05-28 10:00 MSK</t>
+          <t>Wed, 27 Jul 2022 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2886,12 +2886,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://vmo24.ru/news/vadim_lobov_predprinimatel_i_sozdatel_sinergii</t>
+          <t>https://www.forbes.ru/svoi-biznes/472819-korporacia-sinergia-priobrela-cast-rossijskogo-biznesa-mezdunarodnoj-gruppy-hays</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>vmo24.ru</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2913,22 +2913,22 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2025-09-10 10:00 MSK</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2938,12 +2938,12 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2965,22 +2965,22 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>ФШР и Университет "Синергия" заключили соглашение о сотрудничестве</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>SakhaDay</t>
+          <t>Федерация шахмат России</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2024-08-12 10:00 MSK</t>
+          <t>Wed, 11 Sep 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2990,12 +2990,12 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQRjNmbFlVcnA0a0wxTWx2S196aGVlbjVpV2pfUFd0V1BFWXRQTXA3NVRxa1ZWcXFUdlE5M05aR0lkVHRUSDRwQUtsdll1SFZkYkM3WXk2SFRiWVFoekY1MG44MGY5RmQzOEk4NzhDaXl1WThKMGZ0OVBMbWFmMFhBT0lKZUEtbmFxYndyS3FWRFdTb3hyOUZ5SU52UVJCUHpN?oc=5</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -3017,22 +3017,22 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>С Днём рождения, Вадим Лобов!</t>
+          <t>Академическое искусство становится новым трендом</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Союз ММА России</t>
+          <t>The Art Newspaper Russia</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2021-08-02 10:00 MSK</t>
+          <t>Fri, 11 Sep 2026 09:42:00 GMT</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://mmaunion.ru/news/s-dnyom-rozhdeniya-vadim-lobov/</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9HQlF2a05XSW11a3dJSFJZNUtpTTlDRDA4RUpPZXY1YjZlMmJGMFdjZVprMmtES2Q2OV9UdE1qN3FCb1NSeHlrMjNKRFFqbWp2UmtnNFlfbXFHeFRib19IUg?oc=5</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>mmaunion.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -3069,22 +3069,22 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Корпорация «Синергия» приобрела часть российского бизнеса международной группы Hays</t>
+          <t>Posta Art: открытие ярмарки современного искусства «Арт Россия» в Гостином дворе</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Forbes.ru</t>
+          <t>Posta-Magazine</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2022-07-27 10:00 MSK</t>
+          <t>Sat, 05 Apr 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3094,12 +3094,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://www.forbes.ru/svoi-biznes/472819-korporacia-sinergia-priobrela-cast-rossijskogo-biznesa-mezdunarodnoj-gruppy-hays</t>
+          <t>https://posta-magazine.ru/article/art-russia-2025-opening/</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>forbes.ru</t>
+          <t>posta-magazine.ru</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Осетия ТВ</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2024-02-03 11:00 MSK</t>
+          <t>Wed, 10 Sep 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3146,12 +3146,12 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>ossetia.tv</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3173,22 +3173,22 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Posta Art: открытие ярмарки современного искусства «Арт Россия» в Гостином дворе</t>
+          <t>СКР и Корпорация «Синергия» заключили соглашение о сотрудничестве</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Posta-Magazine</t>
+          <t>russkating.ru</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2025-04-05 10:00 MSK</t>
+          <t>Sat, 11 Mar 2023 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3198,12 +3198,12 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://posta-magazine.ru/article/art-russia-2025-opening/</t>
+          <t>https://www.russkating.ru/post/%D1%81%D0%BA%D1%80-%D0%B8-%D0%BA%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F-%D1%81%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F-%D0%B7%D0%B0%D0%BA%D0%BB%D1%8E%D1%87%D0%B8%D0%BB%D0%B8-%D1%81%D0%BE%D0%B3%D0%BB%D0%B0%D1%88%D0%B5%D0%BD%D0%B8%D0%B5-%D0%BE-%D1%81%D0%BE%D1%82%D1%80%D1%83%D0%B4%D0%BD%D0%B8%D1%87%D0%B5%D1%81%D1%82%D0%B2%D0%B5</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>posta-magazine.ru</t>
+          <t>russkating.ru</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -3225,22 +3225,22 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>«Синергия» и Право.ru договорились развивать правовую культуру РФ - новости Право.ру</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>ПРАВО.Ru</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2023-05-11 10:00 MSK</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3250,12 +3250,12 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>https://pravo.ru/lf/news/246443/</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>pravo.ru</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3265,7 +3265,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -3277,22 +3277,22 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>СКР и Корпорация «Синергия» заключили соглашение о сотрудничестве</t>
+          <t>Вадим Георгиевич Лобов: Выход из Болонской системы сохранит кадровые ресурсы России</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>russkating.ru</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2023-03-11 11:00 MSK</t>
+          <t>Wed, 14 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -3302,12 +3302,12 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>https://www.russkating.ru/post/%D1%81%D0%BA%D1%80-%D0%B8-%D0%BA%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F-%D1%81%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F-%D0%B7%D0%B0%D0%BA%D0%BB%D1%8E%D1%87%D0%B8%D0%BB%D0%B8-%D1%81%D0%BE%D0%B3%D0%BB%D0%B0%D1%88%D0%B5%D0%BD%D0%B8%D0%B5-%D0%BE-%D1%81%D0%BE%D1%82%D1%80%D1%83%D0%B4%D0%BD%D0%B8%D1%87%D0%B5%D1%81%D1%82%D0%B2%D0%B5</t>
+          <t>https://megapolisonline.ru/vadim-georgievich-lobov-vyhod-iz-bolonskoj-sistemy-sohranit-kadrovye-resursy-rossii/</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>russkating.ru</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -3329,12 +3329,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Глава «Синергии» Вадим Лобов пригласил участников ВФМ-2024 стать амбассадорами российского образования за рубежом — Осетия ТВ</t>
+          <t>Глава «Синергии» Вадим Лобов анонсировал запуск Центра трансфера технологий для превращения инноваций в бизнес-продукты — Осетия ТВ</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2024-03-09 11:00 MSK</t>
+          <t>Tue, 07 Mar 2023 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2024/03/09/glava-sinergii-vadim-lobov-priglasil-uchastnikov-vfm-2024-stat-ambassadorami-rossijskogo-obrazovaniya-za-rubezhom/</t>
+          <t>https://www.ossetia.tv/2023/03/07/lobov-vadim-georgievich-universiteta-sinergiya/</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -3373,112 +3373,8 @@
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>лобов вадим</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Глава «Синергии» Вадим Лобов объявил о запуске программ двойного диплома с вузами Сербии</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Осетия ТВ</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>2022-08-31 10:00 MSK</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>сниппет Google недоступен</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ossetia.tv/2022/08/31/universitet-sinergiya-serbua/</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>ossetia.tv</t>
-        </is>
-      </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>новость</t>
-        </is>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>лобов вадим</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Глава «Синергии» Вадим Лобов анонсировал запуск Центра трансфера технологий для превращения инноваций в бизнес-продукты — Осетия ТВ</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Осетия ТВ</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>2023-03-07 11:00 MSK</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>сниппет Google недоступен</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ossetia.tv/2023/03/07/lobov-vadim-georgievich-universiteta-sinergiya/</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>ossetia.tv</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>новость (анонс)</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J58"/>
+  <autoFilter ref="A1:J56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Collect the 8 Oct Google News screen and add a summary comparison table.
The Oct snapshot is compared with 13 Sep: 55 to 52 cards, Sostav loses all three #1 slots, and Excel now has a combined sheet with previous/current position and status for every card.

Co-authored-by: Ilya Rost <jaguarcatcat@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/aktualnaya_vydacha.xlsx
+++ b/output/aktualnaya_vydacha.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Выдача" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Выдача'!$A$1:$J$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Выдача'!$A$1:$J$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -526,12 +526,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов и корпорация "Синергия" в фокусе внимания моего очередного подкаста ЖЗЛ Ростокин. Digital</t>
+          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -546,17 +546,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://www.sostav.ru/blogs/289047/94470</t>
+          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>блог / колонка / подкаст</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -578,17 +578,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
+          <t>Вадим Лобов — обо мне</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Сноб</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
+          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
         </is>
       </c>
     </row>
@@ -682,17 +682,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -702,12 +702,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -734,17 +734,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -754,17 +754,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -786,17 +786,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов — обо мне</t>
+          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Сноб</t>
+          <t>Проект медиа</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
+          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -806,22 +806,22 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
+          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>proekt.media</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>расследование</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
         </is>
       </c>
     </row>
@@ -838,17 +838,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -858,22 +858,22 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -890,17 +890,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
+          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Проект медиа</t>
+          <t>Парламент.UA</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
+          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -910,22 +910,22 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
+          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>proekt.media</t>
+          <t>parlament.ua</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>расследование</t>
+          <t>досье / биография</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
         </is>
       </c>
     </row>
@@ -942,17 +942,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Интервью с президентом «Синергии»: «Будем привлекать молодежь к правовому просвещению школьников» - новости Право.ру</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ПРАВО.Ru</t>
+          <t>SakhaDay</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Fri, 05 Jul 2024 07:00:00 GMT</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -962,22 +962,22 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://pravo.ru/story/253963/</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>pravo.ru</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>интервью</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
         </is>
       </c>
     </row>
@@ -994,17 +994,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Парламент.UA</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1014,22 +1014,22 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>parlament.ua</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>досье / биография</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -1046,17 +1046,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>Университет «Синергия»: лох не мамонт – лох заплатит за диплом!</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
+          <t>Fri, 27 May 2022 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNUHpuSllKSUFDX2QtZFlEMG1xdTA2WVc2RDhaak41X3JVZHdGZEtyb0ZNX2VfWWxHNFVYUndBMUZOSDhnQ2tmcm90bmU3dGZFaFdsSUpYNDIycDUzeC14R0lWWUgtUEFQaFdQTWFuR1l1WUZlRmtsTVBJX1ZCdzN0b1ZfSmMxbHIwXzh2TUxSVWZNMXM?oc=5</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия, университет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1098,17 +1098,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов: Наши студенты смогут получить два диплома — «Синергии» и ведущего университета страны БРИКС | Россия-Онлайн- новости России</t>
+          <t>Мошенничество под прикрытием ВУЗа: как разводят на деньги студентов «Синергии»</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>russia-on.ru</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Feb 2024 08:00:00 GMT</t>
+          <t>Fri, 13 Jun 2025 03:11:20 GMT</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiRkFVX3lxTE5rTkNqaHYwV0NDQjUtQVRrazJ4SFV0OXM5dmYzVTctWUxPdzRCc284YVFsM0o4YjBkOFJKY090c3pVbDF3NHc?oc=5</t>
+          <t>https://repost.news/news/11272-moshennichestvo_pod_prikrytiem_vuza_kak_razvodjat_na_denjgi_studentov_sinergii</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1133,34 +1133,34 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим университет синергия</t>
+          <t>лобов вадим синергия</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Глава «Синергии» Вадим Лобов анонсировал запуск Центра трансфера технологий для превращения инноваций в бизнес-продукты — Осетия ТВ</t>
+          <t>Вадим Лобов поделился подробностями проекта по возрождению военной подготовки для молодежи</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>Общественная служба новостей</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Tue, 07 Mar 2023 08:00:00 GMT</t>
+          <t>Mon, 21 Sep 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1170,49 +1170,49 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2023/03/07/lobov-vadim-georgievich-universiteta-sinergiya/</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQcTQzelBmZ3lxekxlOGdSSVNEdV9BYVRtbERlakVMWFJfbkVCQU9DU2NmSFlXaGRreV95TndSS3g2dUd2ZFJHMl9GOUZYWlctUjYzUVI5UnQxaDNtRjhLNG1VMTh4QV9pS1h6TWtXRS1GSXlsRHU5ZVB2c0hMX3QtVHVncG1zRjc1LXo1Y3lxbDhPUlBvOFA5ZnlBY3gxZUlOODFLcDc3aUZpLVdvb092Y3ZwVjJZekk3UHRQU0k0ZU5sVGtSR0pEbndhdW0?oc=5</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим университет синергия</t>
+          <t>лобов вадим синергия</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Президент «Синергии» Лобов: «Грамотная миграционная политика—решение проблемы кадров»</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
+          <t>Mon, 29 Dec 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1222,12 +1222,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://www.forbes.ru/club/552791-prezident-sinergii-lobov-gramotnaa-migracionnaa-politika-resenie-problemy-kadrov</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1237,34 +1237,34 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим университет синергия</t>
+          <t>лобов вадим синергия</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Мошенничество под прикрытием ВУЗа: как разводят на деньги студентов «Синергии»</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Tue, 15 Nov 2022 08:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/11272-moshennichestvo_pod_prikrytiem_vuza_kak_razvodjat_na_denjgi_studentov_sinergii</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1301,22 +1301,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов и корпорация "Синергия" в фокусе внимания моего очередного подкаста ЖЗЛ Ростокин. Digital</t>
+          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>zarya-egorlik.ru</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
+          <t>Tue, 20 Jan 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1326,22 +1326,22 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>https://www.sostav.ru/blogs/289047/94470</t>
+          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>zarya-egorlik.ru</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>блог / колонка / подкаст</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1353,22 +1353,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Президент «Синергии» Лобов: «Грамотная миграционная политика—решение проблемы кадров»</t>
+          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Forbes.ru</t>
+          <t>SMINEWS</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Mon, 29 Dec 2025 08:00:00 GMT</t>
+          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1378,22 +1378,22 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>https://www.forbes.ru/club/552791-prezident-sinergii-lobov-gramotnaa-migracionnaa-politika-resenie-problemy-kadrov</t>
+          <t>https://sminews.ru/2891</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>forbes.ru</t>
+          <t>sminews.ru</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1405,22 +1405,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
+          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Журнал ФОМА</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
+          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>foma.ru</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
         </is>
       </c>
     </row>
@@ -1457,22 +1457,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
+          <t>Вадим Лобов — обо мне</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Журнал ФОМА</t>
+          <t>Сноб</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
+          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1482,12 +1482,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>foma.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -1509,22 +1509,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Президент «Синергии» Лобов представил патриарху Кириллу проект экотроп на Валааме</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Общественная служба новостей</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1534,22 +1534,22 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPS3ZGa1N3RGN2aU9yRkxpT3NKb2Z3RFJ4b3VjbWl6S3V2QmxDU2FSbng3eUdoWm1kQk9OMnNmbU9JeTcxX3VtNC1OSExJTGQ3UllKYkZRZnYtM2kxVV9NOUZ1TFZRNnNmNVdtc3Vnd2k1bzVSeTRxWmFJVGhLY0dpUWhxaVN3cG1nb0Q0b3hDOUhlUmV6RVgxRTlBRmQ2aDd3N21USGJ3X280dXdqRlNoeHFKdzgtZw?oc=5</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1561,22 +1561,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
+          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>SMINEWS</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1586,17 +1586,17 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>https://sminews.ru/2891</t>
+          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>sminews.ru</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1613,22 +1613,22 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
+          <t>Президент «Синергии» Лобов представил патриарху Кириллу проект экотроп на Валааме</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>Общественная служба новостей</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Tue, 20 Jan 2026 08:00:00 GMT</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPS3ZGa1N3RGN2aU9yRkxpT3NKb2Z3RFJ4b3VjbWl6S3V2QmxDU2FSbng3eUdoWm1kQk9OMnNmbU9JeTcxX3VtNC1OSExJTGQ3UllKYkZRZnYtM2kxVV9NOUZ1TFZRNnNmNVdtc3Vnd2k1bzVSeTRxWmFJVGhLY0dpUWhxaVN3cG1nb0Q0b3hDOUhlUmV6RVgxRTlBRmQ2aDd3N21USGJ3X280dXdqRlNoeHFKdzgtZw?oc=5</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
         </is>
       </c>
     </row>
@@ -1665,22 +1665,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов — обо мне</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Сноб</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1717,22 +1717,22 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
+          <t>«Синергия» и Право.ru договорились развивать правовую культуру РФ - новости Право.ру</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>ПРАВО.Ru</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
+          <t>Thu, 11 May 2023 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1742,12 +1742,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
+          <t>https://pravo.ru/lf/news/246443/</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>pravo.ru</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1769,22 +1769,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>Проект медиа</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
+          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1794,22 +1794,22 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>proekt.media</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>расследование</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1821,22 +1821,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>Рост EdTech-выручки «Синергии» трехкратно превысил средний показатель рынка</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>TAdviser</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
+          <t>Fri, 26 Apr 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1846,12 +1846,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://www.tadviser.ru/index.php/%D0%9A%D0%BE%D0%BC%D0%BF%D0%B0%D0%BD%D0%B8%D1%8F:%D0%A1%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F_%D0%9A%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>tadviser.ru</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1873,22 +1873,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Интервью с президентом «Синергии»: «Будем привлекать молодежь к правовому просвещению школьников» - новости Право.ру</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ПРАВО.Ru</t>
+          <t>SakhaDay</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Fri, 05 Jul 2024 07:00:00 GMT</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1898,22 +1898,22 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>https://pravo.ru/story/253963/</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>pravo.ru</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>интервью</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -1925,22 +1925,22 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
+          <t>Предновогодний гала-вечер «Хрустальная симфония» Корпорации «Синергия» и Posta-Magazine</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Проект медиа</t>
+          <t>Posta-Magazine</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
+          <t>Mon, 16 Dec 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1950,17 +1950,17 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
+          <t>https://posta-magazine.ru/article/khrustalnaya-simfonia-2024/</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>proekt.media</t>
+          <t>posta-magazine.ru</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>расследование</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -1977,22 +1977,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>Парламент.UA</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
+          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2002,17 +2002,17 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>parlament.ua</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>досье / биография</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2029,22 +2029,22 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Рост EdTech-выручки «Синергии» трехкратно превысил средний показатель рынка</t>
+          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>TAdviser</t>
+          <t>Осетия ТВ</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Fri, 26 Apr 2024 07:00:00 GMT</t>
+          <t>Wed, 10 Sep 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2054,12 +2054,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>https://www.tadviser.ru/index.php/%D0%9A%D0%BE%D0%BC%D0%BF%D0%B0%D0%BD%D0%B8%D1%8F:%D0%A1%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F_%D0%9A%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F</t>
+          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>tadviser.ru</t>
+          <t>ossetia.tv</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -2081,22 +2081,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Предновогодний гала-вечер «Хрустальная симфония» Корпорации «Синергия» и Posta-Magazine</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Posta-Magazine</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Mon, 16 Dec 2024 08:00:00 GMT</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2106,12 +2106,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>https://posta-magazine.ru/article/khrustalnaya-simfonia-2024/</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>posta-magazine.ru</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2180,27 +2180,27 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим синергия</t>
+          <t>лобов вадим</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Корпорация «Синергия» приобрела часть российского бизнеса международной группы Hays</t>
+          <t>Вадим Лобов поделился подробностями проекта по возрождению военной подготовки для молодежи</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Forbes.ru</t>
+          <t>Общественная служба новостей</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Wed, 27 Jul 2022 07:00:00 GMT</t>
+          <t>Mon, 21 Sep 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2210,12 +2210,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>https://www.forbes.ru/svoi-biznes/472819-korporacia-sinergia-priobrela-cast-rossijskogo-biznesa-mezdunarodnoj-gruppy-hays</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQcTQzelBmZ3lxekxlOGdSSVNEdV9BYVRtbERlakVMWFJfbkVCQU9DU2NmSFlXaGRreV95TndSS3g2dUd2ZFJHMl9GOUZYWlctUjYzUVI5UnQxaDNtRjhLNG1VMTh4QV9pS1h6TWtXRS1GSXlsRHU5ZVB2c0hMX3QtVHVncG1zRjc1LXo1Y3lxbDhPUlBvOFA5ZnlBY3gxZUlOODFLcDc3aUZpLVdvb092Y3ZwVjJZekk3UHRQU0k0ZU5sVGtSR0pEbndhdW0?oc=5</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>forbes.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2225,34 +2225,34 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим синергия</t>
+          <t>лобов вадим</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Основатели «Арт России» Вадим Лобов и Елизавета Фролова — о коллекционировании без посредников</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Buro 24/7</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
+          <t>Fri, 27 Mar 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2262,12 +2262,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://www.buro247.ru/culture/arts/23-mar-2026-art-russia-interview.html</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>buro247.ru</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2277,34 +2277,34 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим синергия</t>
+          <t>лобов вадим</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов: Наши студенты смогут получить два диплома — «Синергии» и ведущего университета страны БРИКС | Россия-Онлайн- новости России</t>
+          <t>Президент «Синергии» Лобов: «Грамотная миграционная политика—решение проблемы кадров»</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>russia-on.ru</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Feb 2024 08:00:00 GMT</t>
+          <t>Mon, 29 Dec 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2314,12 +2314,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiRkFVX3lxTE5rTkNqaHYwV0NDQjUtQVRrazJ4SFV0OXM5dmYzVTctWUxPdzRCc284YVFsM0o4YjBkOFJKY090c3pVbDF3NHc?oc=5</t>
+          <t>https://www.forbes.ru/club/552791-prezident-sinergii-lobov-gramotnaa-migracionnaa-politika-resenie-problemy-kadrov</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов. Не видны: вадим.</t>
         </is>
       </c>
     </row>
@@ -2341,22 +2341,22 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов и корпорация "Синергия" в фокусе внимания моего очередного подкаста ЖЗЛ Ростокин. Digital</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2366,17 +2366,17 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>https://www.sostav.ru/blogs/289047/94470</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>sostav.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>блог / колонка / подкаст</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2393,22 +2393,22 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Основатели «Арт России» Вадим Лобов и Елизавета Фролова — о коллекционировании без посредников</t>
+          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>buro247.ru</t>
+          <t>Журнал ФОМА</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Fri, 27 Mar 2026 07:00:00 GMT</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://www.buro247.ru/culture/arts/23-mar-2026-art-russia-interview.html</t>
+          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>buro247.ru</t>
+          <t>foma.ru</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
+          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Журнал ФОМА</t>
+          <t>SMINEWS</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
+          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2470,22 +2470,22 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
+          <t>https://sminews.ru/2891</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>foma.ru</t>
+          <t>sminews.ru</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2497,22 +2497,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
+          <t>Вадим Лобов — обо мне</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Сноб</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
+          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2549,22 +2549,22 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
+          <t>Тимати с Ивановой, желтый синхрон Агаты и Дранги, кот Базилио Хрусталев: открытие «Арт Россия</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>SMINEWS</t>
+          <t>StarHit</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
+          <t>Fri, 03 Apr 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2574,22 +2574,22 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://sminews.ru/2891</t>
+          <t>https://www.starhit.ru/novosti/timati-vopreki-slukham-ob-izmene-prishel-s-ivanovoi-agata-s-drangoi-v-zheltom-sinkhrone-a-khrustalev-v-obraze-kota-bazilio-otkrytie-art-rossiya-6939626/</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>sminews.ru</t>
+          <t>starhit.ru</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2601,22 +2601,22 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов — обо мне</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Сноб</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2626,17 +2626,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2705,22 +2705,22 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2730,17 +2730,17 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -2757,22 +2757,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Тимати с Ивановой, желтый синхрон Агаты и Дранги, кот Базилио Хрусталев: открытие «Арт Россия</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>StarHit</t>
+          <t>SakhaDay</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Fri, 03 Apr 2026 07:00:00 GMT</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2782,12 +2782,12 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>https://www.starhit.ru/novosti/timati-vopreki-slukham-ob-izmene-prishel-s-ivanovoi-agata-s-drangoi-v-zheltom-sinkhrone-a-khrustalev-v-obraze-kota-bazilio-otkrytie-art-rossiya-6939626/</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>starhit.ru</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2809,22 +2809,22 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>ФШР и Университет "Синергия" заключили соглашение о сотрудничестве</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Федерация шахмат России</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
+          <t>Wed, 11 Sep 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2834,12 +2834,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQRjNmbFlVcnA0a0wxTWx2S196aGVlbjVpV2pfUFd0V1BFWXRQTXA3NVRxa1ZWcXFUdlE5M05aR0lkVHRUSDRwQUtsdll1SFZkYkM3WXk2SFRiWVFoekY1MG44MGY5RmQzOEk4NzhDaXl1WThKMGZ0OVBMbWFmMFhBT0lKZUEtbmFxYndyS3FWRFdTb3hyOUZ5SU52UVJCUHpN?oc=5</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2861,22 +2861,22 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Корпорация «Синергия» приобрела часть российского бизнеса международной группы Hays</t>
+          <t>«Синергия» и Право.ru договорились развивать правовую культуру РФ - новости Право.ру</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Forbes.ru</t>
+          <t>ПРАВО.Ru</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Wed, 27 Jul 2022 07:00:00 GMT</t>
+          <t>Thu, 11 May 2023 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2886,12 +2886,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://www.forbes.ru/svoi-biznes/472819-korporacia-sinergia-priobrela-cast-rossijskogo-biznesa-mezdunarodnoj-gruppy-hays</t>
+          <t>https://pravo.ru/lf/news/246443/</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>forbes.ru</t>
+          <t>pravo.ru</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -2913,22 +2913,22 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>Posta Art: открытие ярмарки современного искусства «Арт Россия» в Гостином дворе</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>Posta-Magazine</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
+          <t>Sat, 05 Apr 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2938,12 +2938,12 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://posta-magazine.ru/article/art-russia-2025-opening/</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>posta-magazine.ru</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2965,22 +2965,22 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>ФШР и Университет "Синергия" заключили соглашение о сотрудничестве</t>
+          <t>Представительство Российского образовательного агентства начало работу в Китае</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Федерация шахмат России</t>
+          <t>ФОНД РУССКИЙ МИР</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Wed, 11 Sep 2024 07:00:00 GMT</t>
+          <t>Fri, 29 May 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQRjNmbFlVcnA0a0wxTWx2S196aGVlbjVpV2pfUFd0V1BFWXRQTXA3NVRxa1ZWcXFUdlE5M05aR0lkVHRUSDRwQUtsdll1SFZkYkM3WXk2SFRiWVFoekY1MG44MGY5RmQzOEk4NzhDaXl1WThKMGZ0OVBMbWFmMFhBT0lKZUEtbmFxYndyS3FWRFdTb3hyOUZ5SU52UVJCUHpN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiSkFVX3lxTE5XczdpdjRHT1VHV01uckZ5RTlnOV92RU83eVhoemllcW9adWYxdFFOVFFVQmJwdjBrR2dnSnNaeVpSSEdhcTVKYXln?oc=5</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3017,22 +3017,22 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Академическое искусство становится новым трендом</t>
+          <t>Корпорация «Синергия» приобрела часть российского бизнеса международной группы Hays</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>The Art Newspaper Russia</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Fri, 11 Sep 2026 09:42:00 GMT</t>
+          <t>Wed, 27 Jul 2022 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9HQlF2a05XSW11a3dJSFJZNUtpTTlDRDA4RUpPZXY1YjZlMmJGMFdjZVprMmtES2Q2OV9UdE1qN3FCb1NSeHlrMjNKRFFqbWp2UmtnNFlfbXFHeFRib19IUg?oc=5</t>
+          <t>https://www.forbes.ru/svoi-biznes/472819-korporacia-sinergia-priobrela-cast-rossijskogo-biznesa-mezdunarodnoj-gruppy-hays</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3069,22 +3069,22 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Posta Art: открытие ярмарки современного искусства «Арт Россия» в Гостином дворе</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Posta-Magazine</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Sat, 05 Apr 2025 07:00:00 GMT</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3094,12 +3094,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://posta-magazine.ru/article/art-russia-2025-opening/</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>posta-magazine.ru</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -3121,22 +3121,22 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
+          <t>Вадим Георгиевич Лобов: Выход из Болонской системы сохранит кадровые ресурсы России</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Wed, 10 Sep 2025 07:00:00 GMT</t>
+          <t>Wed, 14 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3146,12 +3146,12 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
+          <t>https://megapolisonline.ru/vadim-georgievich-lobov-vyhod-iz-bolonskoj-sistemy-sohranit-kadrovye-resursy-rossii/</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3173,22 +3173,22 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>СКР и Корпорация «Синергия» заключили соглашение о сотрудничестве</t>
+          <t>Арт Россия 2024: Вадим Георгиевич Лобов раскрыл самые ожидаемые события ярмарки, которая пройдет весной</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>russkating.ru</t>
+          <t>Осетия ТВ</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Sat, 11 Mar 2023 08:00:00 GMT</t>
+          <t>Wed, 31 Aug 2022 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3198,12 +3198,12 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://www.russkating.ru/post/%D1%81%D0%BA%D1%80-%D0%B8-%D0%BA%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F-%D1%81%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F-%D0%B7%D0%B0%D0%BA%D0%BB%D1%8E%D1%87%D0%B8%D0%BB%D0%B8-%D1%81%D0%BE%D0%B3%D0%BB%D0%B0%D1%88%D0%B5%D0%BD%D0%B8%D0%B5-%D0%BE-%D1%81%D0%BE%D1%82%D1%80%D1%83%D0%B4%D0%BD%D0%B8%D1%87%D0%B5%D1%81%D1%82%D0%B2%D0%B5</t>
+          <t>https://www.ossetia.tv/2022/08/31/art-russia-2024/</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>russkating.ru</t>
+          <t>ossetia.tv</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -3213,168 +3213,12 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>лобов вадим</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>сниппет Google недоступен</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>megapolisonline.ru</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>новость</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
           <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>лобов вадим</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Вадим Георгиевич Лобов: Выход из Болонской системы сохранит кадровые ресурсы России</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 14 Feb 2024 08:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>сниппет Google недоступен</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>https://megapolisonline.ru/vadim-georgievich-lobov-vyhod-iz-bolonskoj-sistemy-sohranit-kadrovye-resursy-rossii/</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>megapolisonline.ru</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>новость</t>
-        </is>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>лобов вадим</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Глава «Синергии» Вадим Лобов анонсировал запуск Центра трансфера технологий для превращения инноваций в бизнес-продукты — Осетия ТВ</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Осетия ТВ</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 07 Mar 2023 08:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>сниппет Google недоступен</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ossetia.tv/2023/03/07/lobov-vadim-georgievich-universiteta-sinergiya/</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>ossetia.tv</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>новость (анонс)</t>
-        </is>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J56"/>
+  <autoFilter ref="A1:J53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Collect the 13 Oct Google News screen and export comparison as XLSX and DOCX.
Future runs write both Excel and Word: current SERP plus a comparison against the previous snapshot. This pass is measured against 8 Oct.

Co-authored-by: Ilya Rost <jaguarcatcat@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/aktualnaya_vydacha.xlsx
+++ b/output/aktualnaya_vydacha.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Выдача" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Выдача" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Выдача'!$A$1:$J$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Выдача'!$A$1:$J$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -630,17 +630,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Tue, 20 Jan 2026 08:00:00 GMT</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия, университет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -682,17 +682,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -702,12 +702,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -734,17 +734,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
+          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Проект медиа</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
+          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -754,22 +754,22 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
+          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>proekt.media</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>расследование</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
         </is>
       </c>
     </row>
@@ -786,17 +786,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Проект медиа</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -806,22 +806,22 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>proekt.media</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>расследование</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -838,17 +838,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>Парламент.UA</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
+          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -858,22 +858,22 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>parlament.ua</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>досье / биография</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
         </is>
       </c>
     </row>
@@ -890,17 +890,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Парламент.UA</t>
+          <t>SakhaDay</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -910,17 +910,17 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>parlament.ua</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>досье / биография</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -942,17 +942,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>SakhaDay</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -962,12 +962,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия, университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
@@ -994,17 +994,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Вадим Лобов и университет «Синергия»: обещания и реальные отзывы студентов</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Парламент.UA</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
+          <t>Tue, 12 Nov 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1014,22 +1014,22 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNLUNDR0JfWTQ4MzBkeEdDNVdMS0xUSFVoa3JxR3g1NS1yUHhmb2huT1BxZmtiX1RZdTI0b3A2TWkyUDk5ZEFsV0ZPVm9CblYxZWhlNjg4UjFVYWJEY0JSUHM2U0o1a3ZvVVRLWWFVTDJxZXVIVEI4MkdMZXJFb3V3eUI4TFFYNDVmNW14MExEWmJSTHFieUdSSm9OSjk5Tlg5eVltemtLRdIBrwFBVV95cUxPRlJFVk5NSzBJVVI4TU5mZTdzaE1Bb3V0Rm53cEJLR2V0aTZKUGk2N09DTVJCaWgwNi01dzE3YVhxMk45dXRiMEhUSDlETmp1aVhZOFM0UDJwREk3bEZ4c0lxRU9ZSl8tdmp3WWNJc0VqUFZwNFRiV0Qxd1hBQXBDb00zRHZ3OGNya1FwVFRjc2dSaVVlUmZjZ25GM0kzR1JvMnNucmh5RzVaa0RTSnZj?oc=5</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>обзор / отзывы</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия, университет. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1098,17 +1098,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Мошенничество под прикрытием ВУЗа: как разводят на деньги студентов «Синергии»</t>
+          <t>Президент Корпорации «Синергия» Вадим Лобов заявил о необходимости правового просвещения молодежи</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Fri, 13 Jun 2025 03:11:20 GMT</t>
+          <t>Fri, 12 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/11272-moshennichestvo_pod_prikrytiem_vuza_kak_razvodjat_na_denjgi_studentov_sinergii</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNa3NObm9iRmsxd1RmMmZzTWFMelY2cEVKU2lEVGVwWWktVEtrUmZQM0RxdExGdTl0N1FOR1NGWHMwUDhvVzM2OVN5bGZONG1uY1NPUHo3cG1BellZeDRvOEVXSXBkeVV2eGYxMFJnOFI5WFpwWGFSaTlYMWFZZDNLcXM4S09uZ25CXzVXSnVHcmZLZkY5UEU4Tmk1bkdNeGowUXVmWHl6aXFUVXpvZ1luMXdGaWRCdENibThnUTNCbGRubElvS1VyamFB?oc=5</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1133,34 +1133,34 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: университет.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим синергия</t>
+          <t>лобов вадим университет синергия</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов поделился подробностями проекта по возрождению военной подготовки для молодежи</t>
+          <t>Мошенничество под прикрытием ВУЗа: как разводят на деньги студентов «Синергии»</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Общественная служба новостей</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 07:00:00 GMT</t>
+          <t>Fri, 13 Jun 2025 03:11:20 GMT</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1170,12 +1170,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQcTQzelBmZ3lxekxlOGdSSVNEdV9BYVRtbERlakVMWFJfbkVCQU9DU2NmSFlXaGRreV95TndSS3g2dUd2ZFJHMl9GOUZYWlctUjYzUVI5UnQxaDNtRjhLNG1VMTh4QV9pS1h6TWtXRS1GSXlsRHU5ZVB2c0hMX3QtVHVncG1zRjc1LXo1Y3lxbDhPUlBvOFA5ZnlBY3gxZUlOODFLcDc3aUZpLVdvb092Y3ZwVjJZekk3UHRQU0k0ZU5sVGtSR0pEbndhdW0?oc=5</t>
+          <t>https://repost.news/news/11272-moshennichestvo_pod_prikrytiem_vuza_kak_razvodjat_na_denjgi_studentov_sinergii</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов, университет.</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1249,22 +1249,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
+          <t>Вадим Лобов поделился подробностями проекта по возрождению военной подготовки для молодежи</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Общественная служба новостей</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
+          <t>Mon, 21 Sep 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQcTQzelBmZ3lxekxlOGdSSVNEdV9BYVRtbERlakVMWFJfbkVCQU9DU2NmSFlXaGRreV95TndSS3g2dUd2ZFJHMl9GOUZYWlctUjYzUVI5UnQxaDNtRjhLNG1VMTh4QV9pS1h6TWtXRS1GSXlsRHU5ZVB2c0hMX3QtVHVncG1zRjc1LXo1Y3lxbDhPUlBvOFA5ZnlBY3gxZUlOODFLcDc3aUZpLVdvb092Y3ZwVjJZekk3UHRQU0k0ZU5sVGtSR0pEbndhdW0?oc=5</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -1301,22 +1301,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Университет «Синергия» помогает ветеранам СВО Ростовской области получить новую профессию и адаптироваться к мирной жизни</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Tue, 20 Jan 2026 08:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1326,12 +1326,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>https://www.zarya-egorlik.ru/universitet-sinergiya-pomogaet-veteranam-svo-rostovskoy-oblasti-poluchit-novuyu-professiyu-i-adaptirovatsya-k-mirnoy-zhizni/</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>zarya-egorlik.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1353,22 +1353,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
+          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>SMINEWS</t>
+          <t>Журнал ФОМА</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1378,22 +1378,22 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>https://sminews.ru/2891</t>
+          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>sminews.ru</t>
+          <t>foma.ru</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
         </is>
       </c>
     </row>
@@ -1405,22 +1405,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
+          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Журнал ФОМА</t>
+          <t>SMINEWS</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
+          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1430,22 +1430,22 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
+          <t>https://sminews.ru/2891</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>foma.ru</t>
+          <t>sminews.ru</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1613,22 +1613,22 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Президент «Синергии» Лобов представил патриарху Кириллу проект экотроп на Валааме</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Общественная служба новостей</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPS3ZGa1N3RGN2aU9yRkxpT3NKb2Z3RFJ4b3VjbWl6S3V2QmxDU2FSbng3eUdoWm1kQk9OMnNmbU9JeTcxX3VtNC1OSExJTGQ3UllKYkZRZnYtM2kxVV9NOUZ1TFZRNnNmNVdtc3Vnd2k1bzVSeTRxWmFJVGhLY0dpUWhxaVN3cG1nb0Q0b3hDOUhlUmV6RVgxRTlBRmQ2aDd3N21USGJ3X280dXdqRlNoeHFKdzgtZw?oc=5</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов, синергия. Не видны: вадим.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -1665,22 +1665,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>«Синергия» и Право.ru договорились развивать правовую культуру РФ - новости Право.ру</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>ПРАВО.Ru</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
+          <t>Thu, 11 May 2023 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://pravo.ru/lf/news/246443/</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>pravo.ru</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1717,22 +1717,22 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>«Синергия» и Право.ru договорились развивать правовую культуру РФ - новости Право.ру</t>
+          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ПРАВО.Ru</t>
+          <t>Проект медиа</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Thu, 11 May 2023 07:00:00 GMT</t>
+          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1742,17 +1742,17 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>https://pravo.ru/lf/news/246443/</t>
+          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>pravo.ru</t>
+          <t>proekt.media</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>расследование</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -1769,22 +1769,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Как устроен бизнес крупнейшего частного вуза "Синергия" • Проект.</t>
+          <t>Рост EdTech-выручки «Синергии» трехкратно превысил средний показатель рынка</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Проект медиа</t>
+          <t>TAdviser</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Mon, 22 Oct 2018 07:00:00 GMT</t>
+          <t>Fri, 26 Apr 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>https://www.proekt.media/investigation/synergiya-biznes/</t>
+          <t>https://www.tadviser.ru/index.php/%D0%9A%D0%BE%D0%BC%D0%BF%D0%B0%D0%BD%D0%B8%D1%8F:%D0%A1%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F_%D0%9A%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>proekt.media</t>
+          <t>tadviser.ru</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>расследование</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -1821,22 +1821,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Рост EdTech-выручки «Синергии» трехкратно превысил средний показатель рынка</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>TAdviser</t>
+          <t>SakhaDay</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Fri, 26 Apr 2024 07:00:00 GMT</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1846,12 +1846,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>https://www.tadviser.ru/index.php/%D0%9A%D0%BE%D0%BC%D0%BF%D0%B0%D0%BD%D0%B8%D1%8F:%D0%A1%D0%B8%D0%BD%D0%B5%D1%80%D0%B3%D0%B8%D1%8F_%D0%9A%D0%BE%D1%80%D0%BF%D0%BE%D1%80%D0%B0%D1%86%D0%B8%D1%8F</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>tadviser.ru</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -1873,22 +1873,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>Предновогодний гала-вечер «Хрустальная симфония» Корпорации «Синергия» и Posta-Magazine</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>SakhaDay</t>
+          <t>Posta-Magazine</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
+          <t>Mon, 16 Dec 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://posta-magazine.ru/article/khrustalnaya-simfonia-2024/</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>posta-magazine.ru</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -1925,22 +1925,22 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Предновогодний гала-вечер «Хрустальная симфония» Корпорации «Синергия» и Posta-Magazine</t>
+          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Posta-Magazine</t>
+          <t>Парламент.UA</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Mon, 16 Dec 2024 08:00:00 GMT</t>
+          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1950,22 +1950,22 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://posta-magazine.ru/article/khrustalnaya-simfonia-2024/</t>
+          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>posta-magazine.ru</t>
+          <t>parlament.ua</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>досье / биография</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -1977,22 +1977,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов - досье, биография, фото, последние новости</t>
+          <t>Корпорация «Синергия» приобрела часть российского бизнеса международной группы Hays</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Парламент.UA</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Thu, 18 Jul 2024 07:00:00 GMT</t>
+          <t>Wed, 27 Jul 2022 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2002,22 +2002,22 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>https://parlament.ua/ru/dossier/lobov-vadim/</t>
+          <t>https://www.forbes.ru/svoi-biznes/472819-korporacia-sinergia-priobrela-cast-rossijskogo-biznesa-mezdunarodnoj-gruppy-hays</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>parlament.ua</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>досье / биография</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
+          <t>Средняя релевантность: есть «Синергия», но персона в заголовке/URL не видна. Совпавшие токены: синергия. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2029,22 +2029,22 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
+          <t>Президент Корпорации «Синергия» Вадим Лобов заявил о необходимости правового просвещения молодежи</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Осетия ТВ</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Wed, 10 Sep 2025 07:00:00 GMT</t>
+          <t>Fri, 12 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2054,12 +2054,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNa3NObm9iRmsxd1RmMmZzTWFMelY2cEVKU2lEVGVwWWktVEtrUmZQM0RxdExGdTl0N1FOR1NGWHMwUDhvVzM2OVN5bGZONG1uY1NPUHo3cG1BellZeDRvOEVXSXBkeVV2eGYxMFJnOFI5WFpwWGFSaTlYMWFZZDNLcXM4S09uZ25CXzVXSnVHcmZLZkY5UEU4Tmk1bkdNeGowUXVmWHl6aXFUVXpvZ1luMXdGaWRCdENibThnUTNCbGRubElvS1VyamFB?oc=5</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>ossetia.tv</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2081,22 +2081,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Осетия ТВ</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
+          <t>Wed, 10 Sep 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2106,12 +2106,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>ossetia.tv</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
+          <t>Средняя релевантность: персона частично совпадает, часть запроса в карточке не видна. Совпавшие токены: вадим, лобов. Не видны: синергия.</t>
         </is>
       </c>
     </row>
@@ -2133,22 +2133,22 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Елизавета Фролова: «Я вижу тренд на возвращение академического искусства»</t>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>The Art Newspaper Russia</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Thu, 18 Sep 2025 07:00:00 GMT</t>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9SX0U3RnB1SmQteFRTNVZJdkRUNmZWWkZlVTdiYUYyUVNMcFdhSFVab1dGa1gzNllPUXdEczRMMnhEeFVGM3I4TkU3Mk05bDk2RU94T21vX2dOU2huVWwxZQ?oc=5</t>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>megapolisonline.ru</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2173,34 +2173,34 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов, синергия.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>лобов вадим</t>
+          <t>лобов вадим синергия</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов поделился подробностями проекта по возрождению военной подготовки для молодежи</t>
+          <t>Вадим Лобов и университет «Синергия»: обещания и реальные отзывы студентов</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Общественная служба новостей</t>
+          <t>Парламент.UA</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 07:00:00 GMT</t>
+          <t>Tue, 12 Nov 2024 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQcTQzelBmZ3lxekxlOGdSSVNEdV9BYVRtbERlakVMWFJfbkVCQU9DU2NmSFlXaGRreV95TndSS3g2dUd2ZFJHMl9GOUZYWlctUjYzUVI5UnQxaDNtRjhLNG1VMTh4QV9pS1h6TWtXRS1GSXlsRHU5ZVB2c0hMX3QtVHVncG1zRjc1LXo1Y3lxbDhPUlBvOFA5ZnlBY3gxZUlOODFLcDc3aUZpLVdvb092Y3ZwVjJZekk3UHRQU0k0ZU5sVGtSR0pEbndhdW0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNLUNDR0JfWTQ4MzBkeEdDNVdMS0xUSFVoa3JxR3g1NS1yUHhmb2huT1BxZmtiX1RZdTI0b3A2TWkyUDk5ZEFsV0ZPVm9CblYxZWhlNjg4UjFVYWJEY0JSUHM2U0o1a3ZvVVRLWWFVTDJxZXVIVEI4MkdMZXJFb3V3eUI4TFFYNDVmNW14MExEWmJSTHFieUdSSm9OSjk5Tlg5eVltemtLRdIBrwFBVV95cUxPRlJFVk5NSzBJVVI4TU5mZTdzaE1Bb3V0Rm53cEJLR2V0aTZKUGk2N09DTVJCaWgwNi01dzE3YVhxMk45dXRiMEhUSDlETmp1aVhZOFM0UDJwREk3bEZ4c0lxRU9ZSl8tdmp3WWNJc0VqUFZwNFRiV0Qxd1hBQXBDb00zRHZ3OGNya1FwVFRjc2dSaVVlUmZjZ25GM0kzR1JvMnNucmh5RzVaa0RTSnZj?oc=5</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2220,12 +2220,12 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>обзор / отзывы</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Высокая релевантность: в карточке есть и персона, и «Синергия». Совпавшие токены: вадим, лобов, синергия. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Президент «Синергии» Лобов: «Грамотная миграционная политика—решение проблемы кадров»</t>
+          <t>Вадим Лобов поделился подробностями проекта по возрождению военной подготовки для молодежи</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Forbes.ru</t>
+          <t>Общественная служба новостей</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Mon, 29 Dec 2025 08:00:00 GMT</t>
+          <t>Mon, 21 Sep 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2314,12 +2314,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>https://www.forbes.ru/club/552791-prezident-sinergii-lobov-gramotnaa-migracionnaa-politika-resenie-problemy-kadrov</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQcTQzelBmZ3lxekxlOGdSSVNEdV9BYVRtbERlakVMWFJfbkVCQU9DU2NmSFlXaGRreV95TndSS3g2dUd2ZFJHMl9GOUZYWlctUjYzUVI5UnQxaDNtRjhLNG1VMTh4QV9pS1h6TWtXRS1GSXlsRHU5ZVB2c0hMX3QtVHVncG1zRjc1LXo1Y3lxbDhPUlBvOFA5ZnlBY3gxZUlOODFLcDc3aUZpLVdvb092Y3ZwVjJZekk3UHRQU0k0ZU5sVGtSR0pEbndhdW0?oc=5</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>forbes.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов. Не видны: вадим.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2341,22 +2341,22 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
+          <t>Президент «Синергии» Лобов: «Грамотная миграционная политика—решение проблемы кадров»</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Forbes.ru</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
+          <t>Mon, 29 Dec 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
+          <t>https://www.forbes.ru/club/552791-prezident-sinergii-lobov-gramotnaa-migracionnaa-politika-resenie-problemy-kadrov</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>forbes.ru</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Высокая релевантность: есть фамилия и «Синергия», имя в карточке может быть опущено. Совпавшие токены: лобов. Не видны: вадим.</t>
         </is>
       </c>
     </row>
@@ -2393,22 +2393,22 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
+          <t>Вадим Лобов и «Синергия» развивают партнерство с Валаамским монастырем</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Журнал ФОМА</t>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNdElGeTNGaldKWnFoeWRLVFB0QzhVTmtYNUVjNktlazZEN0xuNG96WkRQRTdVczAyV2w2dG1aRjFNTkR3TkhZX0E3TVRhR3V5UFdMZUlHZl92c0d5eGJWeEQ5LU1RelEySHZ6cTZ6OGd6NFhPR0ZRMzZEZjM3cnhCcVVzSDRjNG1TeEZNQ1VvZFR5Vk53aEZpVDl2VmhGNkk?oc=5</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>foma.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
+          <t>они свяжут главные точки обители в единую маршрутную сеть для паломников</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>SMINEWS</t>
+          <t>Журнал ФОМА</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
+          <t>Wed, 15 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2470,22 +2470,22 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>https://sminews.ru/2891</t>
+          <t>https://foma.ru/patriarhu-kirillu-predstavili-proekt-ekotrop-na-valaame-oni-svyazhut-glavnye-tochki-obiteli-v-edinuyu-marshrutnuyu-set-dlya-palomnikov.html</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>sminews.ru</t>
+          <t>foma.ru</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2497,22 +2497,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов — обо мне</t>
+          <t>Вадим Лобов и корпорация «Синергия» запустили выставку «За тридевять земель» на ВДНХ как новое прочтение классики русского искусства с поддержкой мультимедиа форматов — SMINEWS</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Сноб</t>
+          <t>SMINEWS</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
+          <t>Mon, 03 Nov 2025 08:00:00 GMT</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2522,17 +2522,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
+          <t>https://sminews.ru/2891</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>sminews.ru</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2549,22 +2549,22 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Тимати с Ивановой, желтый синхрон Агаты и Дранги, кот Базилио Хрусталев: открытие «Арт Россия</t>
+          <t>Вадим Лобов — обо мне</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>StarHit</t>
+          <t>Сноб</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Fri, 03 Apr 2026 07:00:00 GMT</t>
+          <t>Thu, 08 Feb 2024 07:55:28 GMT</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2574,12 +2574,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://www.starhit.ru/novosti/timati-vopreki-slukham-ob-izmene-prishel-s-ivanovoi-agata-s-drangoi-v-zheltom-sinkhrone-a-khrustalev-v-obraze-kota-bazilio-otkrytie-art-rossiya-6939626/</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE1kcXB5MFZlR0ZVeElLY01UQkZxMklzTkt3UWxHVDZsZmt5STRvSThjbDhEcWdXNmRaZHpBUVhHaGxyUDg5bEdqUWhrUXA?oc=5</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>starhit.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2601,22 +2601,22 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
+          <t>Тимати с Ивановой, желтый синхрон Агаты и Дранги, кот Базилио Хрусталев: открытие «Арт Россия</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Отдел N</t>
+          <t>StarHit</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
+          <t>Fri, 03 Apr 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2626,22 +2626,22 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
+          <t>https://www.starhit.ru/novosti/timati-vopreki-slukham-ob-izmene-prishel-s-ivanovoi-agata-s-drangoi-v-zheltom-sinkhrone-a-khrustalev-v-obraze-kota-bazilio-otkrytie-art-rossiya-6939626/</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>otdeln.ru</t>
+          <t>starhit.ru</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>новость (анонс)</t>
+          <t>новость</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
         </is>
       </c>
     </row>
@@ -2653,22 +2653,22 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
+          <t>Вадим Лобов как президент корпорации Синергия сообщил о создании Центра русского языка в Ираке</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>Отдел N</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
+          <t>Sat, 01 Nov 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2678,17 +2678,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
+          <t>https://otdeln.ru/education/2025/11/01/vadim-lobov-kak-prezident-korporacii-sinergiya-soobshhil-o-sozdanii-centra-russkogo-yazyka-v-irake/</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>nabludatel.od.ua</t>
+          <t>otdeln.ru</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>новость</t>
+          <t>новость (анонс)</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -2705,22 +2705,22 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
+          <t>Лобов Вадим Георгиевич выдоил миллиарды, прикрываясь «Синергией» и физиономией рэпера Басты</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Портал РЕПОСТ</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
+          <t>Mon, 06 Jul 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2730,12 +2730,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
+          <t>https://nabludatel.od.ua/odessa/lobov-vadim-georgievich-i-sinergiya/</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>repost.news</t>
+          <t>nabludatel.od.ua</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2757,22 +2757,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
+          <t>Шарашкин «университет Синергия» и его мошенник-собственник Вадим Лобов озолотится на уклонистах и халтурщиках</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>SakhaDay</t>
+          <t>Портал РЕПОСТ</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
+          <t>Fri, 12 Jul 2024 12:04:18 GMT</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2782,12 +2782,12 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
+          <t>https://repost.news/news/12722-sharashkin_universitet_sinergija_i_ego_moshennik-sobstvennik_vadim_lobov_ozolotitsja_na_uklonistah_i_halturshchikah</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>sakhaday.ru</t>
+          <t>repost.news</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2809,22 +2809,22 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>ФШР и Университет "Синергия" заключили соглашение о сотрудничестве</t>
+          <t>Вадим Лобов: «Якутский колледж цифровых профессий поможет республике готовить кадры для креативной экономики»</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Федерация шахмат России</t>
+          <t>SakhaDay</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Wed, 11 Sep 2024 07:00:00 GMT</t>
+          <t>Mon, 12 Aug 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2834,12 +2834,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQRjNmbFlVcnA0a0wxTWx2S196aGVlbjVpV2pfUFd0V1BFWXRQTXA3NVRxa1ZWcXFUdlE5M05aR0lkVHRUSDRwQUtsdll1SFZkYkM3WXk2SFRiWVFoekY1MG44MGY5RmQzOEk4NzhDaXl1WThKMGZ0OVBMbWFmMFhBT0lKZUEtbmFxYndyS3FWRFdTb3hyOUZ5SU52UVJCUHpN?oc=5</t>
+          <t>https://sakhaday.ru/news/vadim-lobov-yakutskiy-kolledzh-cifrovyh-professiy-pomozhet-respublike-gotovit-kadry-dlya-kreativnoy-ekonomiki</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>sakhaday.ru</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2965,22 +2965,22 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Представительство Российского образовательного агентства начало работу в Китае</t>
+          <t>Выставка «За тридевять земель»: мультимедийное погружение в шедевры русского искусства на ВДНХ при поддержке Вадима Лобова — Осетия ТВ</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>ФОНД РУССКИЙ МИР</t>
+          <t>Осетия ТВ</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Fri, 29 May 2026 07:00:00 GMT</t>
+          <t>Wed, 10 Sep 2025 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2990,12 +2990,12 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiSkFVX3lxTE5XczdpdjRHT1VHV01uckZ5RTlnOV92RU83eVhoemllcW9adWYxdFFOVFFVQmJwdjBrR2dnSnNaeVpSSEdhcTVKYXln?oc=5</t>
+          <t>https://www.ossetia.tv/2025/09/10/vystavka-za-tridevyat-zemel-multimedijnoe-pogruzhenie-v-shedevry-russkogo-iskusstva-na-vdnh-pri-podderzhke-vadima-lobova/</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>news.google.com</t>
+          <t>ossetia.tv</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Низкая релевантность: по видимым полям карточки запрос почти не подтверждается. Совпавшие токены: нет. Не видны: вадим, лобов.</t>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -3069,12 +3069,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+          <t>Президент Корпорации «Синергия» Вадим Лобов заявил о необходимости правового просвещения молодежи</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
+          <t>Fri, 12 Jul 2024 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3094,12 +3094,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNa3NObm9iRmsxd1RmMmZzTWFMelY2cEVKU2lEVGVwWWktVEtrUmZQM0RxdExGdTl0N1FOR1NGWHMwUDhvVzM2OVN5bGZONG1uY1NPUHo3cG1BellZeDRvOEVXSXBkeVV2eGYxMFJnOFI5WFpwWGFSaTlYMWFZZDNLcXM4S09uZ25CXzVXSnVHcmZLZkY5UEU4Tmk1bkdNeGowUXVmWHl6aXFUVXpvZ1luMXdGaWRCdENibThnUTNCbGRubElvS1VyamFB?oc=5</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Вадим Георгиевич Лобов: Выход из Болонской системы сохранит кадровые ресурсы России</t>
+          <t>Арт Россия 2024: Вадим Георгиевич Лобов раскрыл самые ожидаемые события ярмарки, которая пройдет весной</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+          <t>Осетия ТВ</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Wed, 14 Feb 2024 08:00:00 GMT</t>
+          <t>Wed, 31 Aug 2022 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3146,12 +3146,12 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://megapolisonline.ru/vadim-georgievich-lobov-vyhod-iz-bolonskoj-sistemy-sohranit-kadrovye-resursy-rossii/</t>
+          <t>https://www.ossetia.tv/2022/08/31/art-russia-2024/</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>megapolisonline.ru</t>
+          <t>ossetia.tv</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3173,52 +3173,104 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Президент корпорации Синергия Вадим Георгиевич Лобов объявил о выходе на образовательный рынок Африки</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Sat, 03 Feb 2024 08:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>сниппет Google недоступен</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolisonline.ru/prezident-korporatsii-sinergiya-vadim-georgievich-lobov-obyavil-o-vyhode-na-obrazovatelnyj-rynok-afriki/</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>megapolisonline.ru</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>новость</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>лобов вадим</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Арт Россия 2024: Вадим Георгиевич Лобов раскрыл самые ожидаемые события ярмарки, которая пройдет весной</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Осетия ТВ</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 31 Aug 2022 07:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>сниппет Google недоступен</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ossetia.tv/2022/08/31/art-russia-2024/</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>ossetia.tv</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>новость</t>
-        </is>
-      </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Вадим Георгиевич Лобов: Выход из Болонской системы сохранит кадровые ресурсы России</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Мегаполис — Городская сеть информирования и взаимопомощи</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Wed, 14 Feb 2024 08:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>сниппет Google недоступен</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolisonline.ru/vadim-georgievich-lobov-vyhod-iz-bolonskoj-sistemy-sohranit-kadrovye-resursy-rossii/</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>megapolisonline.ru</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>новость</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
         <is>
           <t>Высокая релевантность: в карточке явно фигурируют фамилия и имя. Совпавшие токены: вадим, лобов. Не видны: нет.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J53"/>
+  <autoFilter ref="A1:J54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>